<commit_message>
Inverse 2026 pour utiliser Old dans le frontend
</commit_message>
<xml_diff>
--- a/web/static/documents/achats_siret_fichier_exemple_ma_cantine.xlsx
+++ b/web/static/documents/achats_siret_fichier_exemple_ma_cantine.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="achats_siret_fichier_exemple_ma" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="achats_fichier_exemple_ma_canti" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="35">
   <si>
     <t xml:space="preserve">siret</t>
   </si>
@@ -40,28 +40,91 @@
     <t xml:space="preserve">famille_produits</t>
   </si>
   <si>
-    <t xml:space="preserve">caracteristiques</t>
+    <t xml:space="preserve">categories_egalim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">origine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">est_circuit_court</t>
+  </si>
+  <si>
+    <t xml:space="preserve">est_local</t>
   </si>
   <si>
     <t xml:space="preserve">definition_local</t>
   </si>
   <si>
-    <t xml:space="preserve">Pommes, rouges</t>
+    <t xml:space="preserve">Pommes</t>
   </si>
   <si>
     <t xml:space="preserve">Le bon traiteur</t>
   </si>
   <si>
-    <t xml:space="preserve">90.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTRES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BIO,LOCAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEPARTEMENT</t>
+    <t xml:space="preserve">100.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRUITS_ET_LEGUMES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIO,COMMERCE_EQUITABLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRANCE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REGION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HVE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUROPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poulet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">349.98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VIANDES_VOLAILLES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LABEL_ROUGE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saumon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19.02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRODUITS_DE_LA_MER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PECHE_DURABLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerises</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les fruits rouges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fraises</t>
   </si>
 </sst>
 </file>
@@ -77,6 +140,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -136,13 +200,45 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -268,69 +364,231 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="6.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="14.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="27.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="38.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="21.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="13.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="15.64"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="12" style="2" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" customFormat="false" ht="12.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
-        <v>21010034300016</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="1" t="n">
-        <v>44683</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="0" t="s">
+    <row r="2" customFormat="false" ht="12.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="n">
+        <v>21390218200020</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="C2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="D2" s="6" t="n">
+        <v>46194</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>13</v>
       </c>
+      <c r="F2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="n">
+        <v>21390218200020</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>46195</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="7"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="n">
+        <v>21390218200020</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>46194</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="7"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="n">
+        <v>21390218200020</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>46193</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="7"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="n">
+        <v>21390218200020</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>46193</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="7"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="n">
+        <v>21390218200020</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>46192</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="9"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="7"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>